<commit_message>
Correct the shirt claims: it has not been worn in public yet
Five letters said 'I have been walking the boardwalk in a shirt...' and two
went further and asserted results — 'parents actually ask,' 'strangers ask.'
None of that had happened. Same failure mode as the deal-master story: a claim
running ahead of the facts, in copy aimed at people who could check.

All five now say 'I have had a shirt printed,' which is true. The Browseabout
letter is better for it — the flaw in the plan is the joke, and a plan is
allowed to have a flaw before it has a result.

Audit records that when the shirt is actually worn, the count of people who
stop him is the thing worth putting in letters. A hook tested on strangers is
a claim almost no author can make. Not before there is a number.
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -26111,12 +26111,12 @@
         </is>
       </c>
       <c r="I646" s="5" t="n">
-        <v>1687</v>
+        <v>1685</v>
       </c>
       <c r="J646" s="5" t="inlineStr">
         <is>
           <t>Mr. Keen — congratulations on the building. You took over a school in a town where I spend a good part of my year, so this is a local letter, and I'll keep it short because it's your first fall.
-You may have seen me on the boardwalk this summer in a shirt reading PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Half your families were on that boardwalk in July, mid-negotiation with a seven-year-old over a claw machine. That is the moment this book is about.
+I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, so you may yet see me in it. Half your families were on that boardwalk in July, mid-negotiation with a seven-year-old over a claw machine. That is the moment this book is about.
 I wrote and illustrated a children's book about money. Clarence Gets a Bargain — 36 pages, grades 1-5, and it does the one thing the rest of the category skips. Every other kids' money book teaches saving. Mine teaches a purchase: a boy earns a robot, reads the sale ads at his kitchen table, compares two on a shelf, walks past the newer one deliberately, redeems a coupon at the register, and gets ambushed by sales tax. He is not thrilled about the sales tax. Neither was I at that age.
 Delaware has had K-12 financial literacy standards since 2018, and HB 203 last October sent the whole rollout to high school. Your grade band has the standard and none of the shopping list.
 The teacher side is free — four 45-minute lessons, a discussion guide, assessments with the answer keys already done, and a crosswalk to Jump$tart, CEE, Common Core, and FDIC Money Smart. It prints straight from a browser. No account, no email gate, no cost to the building.
@@ -26638,12 +26638,12 @@
         </is>
       </c>
       <c r="I655" s="5" t="n">
-        <v>1479</v>
+        <v>1482</v>
       </c>
       <c r="J655" s="5" t="inlineStr">
         <is>
           <t>Attn: Leslie Glenn, Youth Services
-Ms. Glenn — I have been walking the boardwalk in a shirt that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. It is either marketing or a cry for help. Strangers keep asking, which was the idea, so I am now asking you.
+Ms. Glenn — I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. It is either marketing or a cry for help, and I intend to find out on the boardwalk this summer. In the meantime I am asking you.
 I wrote and illustrated a children's book and I would like to read it in your building.
 Clarence Gets a Bargain is 36 pages, ages 6-10. A boy earns a robot for good grades and chores, learns to read the sale ads, compares two models in a store, picks the discounted one over the newest one, hands a coupon to a cashier, and discovers sales tax the way we all did — badly, and in public. It reads aloud in about twenty minutes.
 What makes it work for a summer program is that the kids do something afterward. I bring printable mock price tags and ten-percent-off coupons, and there's an online pretend register they can run on a library computer where they ring up the same purchase and watch a markdown and a coupon change the total. It's a book event that turns into an activity without a worksheet in it.
@@ -26697,12 +26697,12 @@
         </is>
       </c>
       <c r="I656" s="5" t="n">
-        <v>1481</v>
+        <v>1530</v>
       </c>
       <c r="J656" s="5" t="inlineStr">
         <is>
           <t>Ms. Noonan — you coordinate the children's programming at Lewes, so you already know the difference between a book event that fills a room and one where six kids show up because it was raining. I'll tell you which one I think this is and you can decide.
-For calibration: I have been walking the boardwalk in a shirt that says PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Parents actually ask. Turns out the arcade is where the money conversation happens whether anybody planned it or not.
+For calibration, I have had a shirt printed that says PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Whether anyone stops me is still an open question. But the arcade is where the money conversation happens whether a parent planned it or not, and that is the whole subject of the book.
 I wrote and illustrated Clarence Gets a Bargain — 36 pages, ages 6-10. A boy earns a robot, does his "shopping homework" in the newspaper sale inserts, compares two models in a store, chooses the cheaper of the two on purpose, redeems a coupon at the checkout, and then meets sales tax and takes it as a personal betrayal. Twenty minutes read aloud.
 The reason it works as programming rather than just a reading: afterward the kids run the purchase themselves. There's a pretend register that runs in any browser, plus printable price tags and coupons, and they figure out the markdown and the discount with their own hands. Seven-year-olds get competitive about it. Loudly.
 No fee. I'm nearby a good part of the year, and I illustrated the book myself, so a drawing session is on the table if that suits the room better.
@@ -26807,11 +26807,11 @@
         </is>
       </c>
       <c r="I658" s="5" t="n">
-        <v>1915</v>
+        <v>1938</v>
       </c>
       <c r="J658" s="5" t="inlineStr">
         <is>
-          <t>James — I have been walking up and down the boardwalk this summer in a shirt that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Strangers ask. I then point them toward a book you do not carry, which is a marketing plan with an obvious flaw in it. Your front door is four blocks from where I am standing when it happens.
+          <t>James — I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, and the plan is to wear it up and down the boardwalk until somebody asks. At which point I will point them toward a book you do not carry. Your front door is four blocks from where I will be standing, so you can see the flaw in my plan as clearly as I can.
 I wrote and illustrated Clarence Gets a Bargain. Thirty-six pages, ages 6-10, hardbound. A boy earns a robot for chores and grades, works the sale ads at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, and then meets sales tax and regards it as a personal insult. Every other children's money book teaches saving. This one teaches the part where a kid is actually standing at a register holding money.
 Two reasons to talk to me rather than the next local author with a tote bag.
 The first is that it is not a signing. Signings are four people and a folding table. I bring printable mock price tags, ten-percent-off coupons, and a pretend register the kids run in a browser, ringing up the same purchase and watching the markdown and the coupon move the total. They get competitive about it. Loudly. Parents stand behind them and read the back cover, which is the actual mechanism.
@@ -26862,7 +26862,7 @@
         </is>
       </c>
       <c r="I659" s="5" t="n">
-        <v>1437</v>
+        <v>1440</v>
       </c>
       <c r="J659" s="5" t="inlineStr">
         <is>
@@ -26870,7 +26870,7 @@
 I would like a table, and I think I fit the ten-to-one o'clock block better than most authors who ask.
 I wrote and illustrated Clarence Gets a Bargain, a 36-page picture book for ages 6-10 about the money skill nobody writes for children: spending. A boy earns a robot, reads the sale ads, compares two models, takes the cheaper one deliberately, redeems a coupon, and discovers sales tax the way we all did, which is badly and in public.
 Here is why the format suits you. Your morning block puts local author talks next to craft vendors, which means families are already circulating and looking for something a child can do with their hands. I am not asking to give a talk. I want a table where kids ring up a purchase themselves — printable price tags, ten-percent-off coupons, and a pretend register running in a browser where a markdown and a coupon visibly change the total. It behaves like a craft table and teaches percentages by accident.
-I am local for a good part of the year. I have also spent this summer walking the boardwalk in a shirt reading PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, which is a fair description of the demand for this at the beach in April.
+I am local for a good part of the year. I have also had a shirt printed reading PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, which I offer less as a credential than as a fair description of the demand for this at the beach in April.
 What is the application, and when does the slate close?
 Jonathan Bach
 Baltimore and Rehoboth Beach

</xml_diff>

<commit_message>
Mark the Browseabout letter DO NOT SEND
They declined the book without reading it, on the basis that someone there
believed she saw AI in a small thumbnail of the cover — which is Jonathan's own
mixed-media illustration. The letter I wrote opens warm and assumes no history,
so to someone who already said no it reads as amnesia or pressure. Kept for
reference inside a collapsed block, flagged at the top of the file, and marked
DEAD in the workbook so it cannot go out by accident.

Two consequences recorded. The Beachside Book Festival is run by Sussex County
Libraries in partnership with Browseabout, so letter 18's cold route could land
in front of the same person — Leslie Glenn is now the required first step
rather than the preferred one. And if one bookseller called AI on a thumbnail,
others will: the art provenance needs to exist in the press kit before the next
person asks, not after.

Ranked three options for Browseabout itself, leading with leaving it alone.
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -26782,12 +26782,12 @@
       </c>
       <c r="C658" s="5" t="inlineStr">
         <is>
-          <t>James Wilson — Browseabout Books</t>
+          <t>Browseabout Books — ⛔ DO NOT SEND</t>
         </is>
       </c>
       <c r="D658" s="5" t="inlineStr">
         <is>
-          <t>Events Coordinator, Browseabout Books</t>
+          <t>They already rejected the book.</t>
         </is>
       </c>
       <c r="E658" s="5" t="inlineStr"/>
@@ -26826,10 +26826,14 @@
       <c r="K658" s="5" t="inlineStr"/>
       <c r="L658" s="5" t="inlineStr">
         <is>
-          <t>Now. Summer is their season and a kids' event needs lead time.</t>
-        </is>
-      </c>
-      <c r="M658" s="5" t="inlineStr"/>
+          <t>⛔ DO NOT SEND — already declined the book without reading it (AI alleged from a cover thumbnail). See letters-delaware.md #17.</t>
+        </is>
+      </c>
+      <c r="M658" s="5" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
       <c r="N658" s="5" t="inlineStr"/>
     </row>
     <row r="659">

</xml_diff>

<commit_message>
Settle the claw-machine figures and put them in the Delaware letters
Confirmed: $25 into the machine, a basketball, $9.99 at Walmart. The recalled
version — a dollar a try, sixteen tries, a ten-dollar toy — was a guess and is
retired. The phrasebank now carries one set of figures with no alternative to
blend it with.

Added to the three Delaware letters that already carried the boardwalk-shirt
line with a claw machine mentioned and no payoff attached. The shirt says ASK
ME HOW; until now nothing in those letters answered it. Left the Browseabout
and April-at-the-beach letters alone — both close on a joke that works, and
arithmetic would flatten them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bCVQmU5dQHBfkG189ujSG
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -26507,12 +26507,12 @@
         </is>
       </c>
       <c r="I646" s="5" t="n">
-        <v>1949</v>
+        <v>2063</v>
       </c>
       <c r="J646" s="5" t="inlineStr">
         <is>
           <t>Mr. Keen — congratulations on the building. You took over a school in a town where I spend a good part of my year, so this is a local letter, and I'll keep it short because it's your first fall.
-I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, so you may yet see me in it. Half your families were on that boardwalk in July, mid-negotiation with a seven-year-old over a claw machine. That is the moment this book is about.
+I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW, so you may yet see me in it. Half your families were on that boardwalk in July, mid-negotiation with a seven-year-old over a claw machine. That machine takes $25 to hand back a basketball Walmart sells for $9.99, and the kid has no way of knowing that. That is the moment this book is about.
 I wrote and illustrated a children's book about money. Clarence Gets a Bargain — 36 pages, grades 1-5, and it does the one thing the rest of the category skips. Every other kids' money book teaches saving. Mine teaches a purchase: a boy earns a robot, reads the sale ads at his kitchen table, compares two on a shelf, walks past the newer one deliberately, redeems a coupon at the register, and gets ambushed by sales tax. He is not thrilled about the sales tax. Neither was I at that age.
 Delaware has had K-12 financial literacy standards since 2018, and HB 203 last October sent the whole rollout to high school. Your grade band has the standard and none of the shopping list.
 The teacher side is free — four 45-minute lessons, a discussion guide, assessments with the answer keys already done, and a crosswalk to Jump$tart, CEE, Common Core, and FDIC Money Smart. It prints straight from a browser. No account, no email gate, no cost to the building.
@@ -27043,12 +27043,12 @@
         </is>
       </c>
       <c r="I655" s="5" t="n">
-        <v>1718</v>
+        <v>1888</v>
       </c>
       <c r="J655" s="5" t="inlineStr">
         <is>
           <t>Attn: Leslie Glenn, Youth Services
-Ms. Glenn — I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. It is either marketing or a cry for help, and I intend to find out on the boardwalk this summer. In the meantime I am asking you.
+Ms. Glenn — I have had a shirt printed that reads PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. It is either marketing or a cry for help, and I intend to find out on the boardwalk this summer. If anyone does ask, the answer is short: the claw machine takes $25 to hand back a basketball Walmart sells for $9.99, and a kid who has seen the $9.99 stops feeding it. In the meantime I am asking you.
 I wrote and illustrated a children's book and I would like to read it in your building.
 Clarence Gets a Bargain is 36 pages, ages 6-10. A boy earns a robot for good grades and chores, learns to read the sale ads, compares two models in a store, picks the discounted one over the newest one, hands a coupon to a cashier, and discovers sales tax the way we all did — badly, and in public. It reads aloud in about twenty minutes.
 What makes it work for a summer program is that the kids do something afterward. I bring printable mock price tags and ten-percent-off coupons, and there's an online pretend register they can run on a library computer where they ring up the same purchase and watch a markdown and a coupon change the total. It's a book event that turns into an activity without a worksheet in it.
@@ -27103,12 +27103,12 @@
         </is>
       </c>
       <c r="I656" s="5" t="n">
-        <v>1766</v>
+        <v>1831</v>
       </c>
       <c r="J656" s="5" t="inlineStr">
         <is>
           <t>Ms. Noonan — you coordinate the children's programming at Lewes, so you already know the difference between a book event that fills a room and one where six kids show up because it was raining. I'll tell you which one I think this is and you can decide.
-For calibration, I have had a shirt printed that says PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Whether anyone stops me is still an open question. But the arcade is where the money conversation happens whether a parent planned it or not, and that is the whole subject of the book.
+For calibration, I have had a shirt printed that says PREVENT BOARDWALK MELTDOWNS &amp; ARCADE HISSY-FITS, ASK ME HOW. Whether anyone stops me is still an open question. But the arcade is where the money conversation happens whether a parent planned it or not — $25 into a glass box for a basketball Walmart sells for $9.99 — and that is the whole subject of the book.
 I wrote and illustrated Clarence Gets a Bargain — 36 pages, ages 6-10. A boy earns a robot, does his "shopping homework" in the newspaper sale inserts, compares two models in a store, chooses the cheaper of the two on purpose, redeems a coupon at the checkout, and then meets sales tax and takes it as a personal betrayal. Twenty minutes read aloud.
 The reason it works as programming rather than just a reading: afterward the kids run the purchase themselves. There's a pretend register that runs in any browser, plus printable price tags and coupons, and they figure out the markdown and the discount with their own hands. Seven-year-olds get competitive about it. Loudly.
 No fee. I'm nearby a good part of the year, and I illustrated the book myself, so a drawing session is on the table if that suits the room better.

</xml_diff>

<commit_message>
Restore the em dashes; make the ruling permanent in CLAUDE.md
I thinned em dashes in ten letters on the strength of a line in CLAUDE.md that
called density an AI tell. Jonathan's ruling: "I support em dashes. They are a
middle finger taking a nap to me." That settles it.

Rebuilt all three letter files from the pre-thinning commit and re-applied only
the two edits worth keeping — twelve kill-list term fixes and twenty-nine
semicolons. Em dashes are back untouched: 203 in the whales, 123 in the top 25,
38 in the grandparent letters.

Replaced the em-dash paranoia entry in CLAUDE.md with the ruling, so no future
pass counts, flags or reduces them. The tells are the never-say terms and the
structural patterns, not punctuation the author has claimed.

Audit stands at one flagged phrase across all 74 letters, kept on purpose
because it is his own recovered sentence.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bCVQmU5dQHBfkG189ujSG
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -994,9 +994,9 @@
           <t>Kim — you review children's books for a living, so you have read more well-meaning money picture books than anyone should have to, and you already know the problem with them.
 They all teach saving. A piggy bank, a lemonade stand, a lesson. Which is fine advice in the wrong order, because saving is the second thing a child does with money; the first is spending. A six-year-old has no savings rate and has absolutely stood in a store holding money and had to decide.
 Mine is the spending one, and it follows a single purchase the whole distance rather than gesturing at the idea: a boy wants a robot, earns it with chores and grades, works the sale ads at the kitchen table, compares two models in the aisle, takes the cheaper one on purpose, hands a coupon to the cashier, gets hit with sales tax, and then has to live with the thing. Idea to post-receipt. I read all 25 on the ABA Foundation's list to be sure nobody had done it. Nobody had.
-What I'd actually want your eye on is the smuggling. Sixteen-plus concepts and not one of them is announced , no character stops to explain a term, nobody says "budget." The reader does not know he's been schooled until he reaches the glossary , twenty-one terms, each page-referenced to the scene it came from, working as a decoder rather than a homework appendix. The reveal is deliberate and it is on the last page. That balance is the hardest thing in the book and the thing most likely to be off by a hair.
+What I'd actually want your eye on is the smuggling. Sixteen-plus concepts and not one of them is announced — no character stops to explain a term, nobody says "budget." The reader does not know he's been schooled until he reaches the glossary — twenty-one terms, each page-referenced to the scene it came from, working as a decoder rather than a homework appendix. The reveal is deliberate and it is on the last page. That balance is the hardest thing in the book and the thing most likely to be off by a hair.
 One thing I'd want you to test rather than take on faith: whether it clicks later. The book is built to fire back months on, in a real store — "is the newer one really better? Clarence checked." Recognition first, then the habit. If that isn't actually in the pages, I'd want to know.
-The other thing worth your reviewer's ear: it is built to be read aloud, and Lexile has it at AD 620L — Adult Directed, read-with rather than read-alone. The mother carries the exposition, which means the adult holding the book is handed the script. Whether that voice actually holds up out loud , across a classroom, a couch, and a grandparent's lap , is something you would hear in a page and I can only guess at.
+The other thing worth your reviewer's ear: it is built to be read aloud, and Lexile has it at AD 620L — Adult Directed, read-with rather than read-alone. The mother carries the exposition, which means the adult holding the book is handed the script. Whether that voice actually holds up out loud — across a classroom, a couch, and a grandparent's lap — is something you would hear in a page and I can only guess at.
 Would you read it as an editor rather than as a friend? I would rather hear where it sags than be told it's charming.
 clarencegetsabargain.com/press-kit.html · https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -1238,9 +1238,9 @@
         <is>
           <t>Cinders — Moneybunnies splits money into Earn, Save, Spend and Give, which makes you the one person in this category who already agreed with me before I showed up.
 I went deep on one of your four. Spending, and specifically the whole transaction rather than the idea of it. Clarence Gets a Bargain follows a single purchase from beginning to end: a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then has to live with what he picked. Idea to post-receipt.
-The reason I think it sits beside Moneybunnies rather than against it: you give a child the four categories, and mine walks them through the mechanics of one. Sixteen-plus concepts, none announced , nobody says "budget" , and twenty-one terms in a glossary in the back, each page-referenced to the scene where it happened.
+The reason I think it sits beside Moneybunnies rather than against it: you give a child the four categories, and mine walks them through the mechanics of one. Sixteen-plus concepts, none announced — nobody says "budget" — and twenty-one terms in a glossary in the back, each page-referenced to the scene where it happened.
 Author-illustrator to author-illustrator: I did the art as well, so I know exactly how much of the work nobody sees. I'd rather you saw this from me than off a shelf.
-The read-aloud is the other half of it. Lexile AD 620L , Adult Directed , written for the adult voice in the room rather than for a child alone, with the mother carrying the explanations so the grown-up gets handed the script. You will know better than most how much that changes what has to happen on the page.
+The read-aloud is the other half of it. Lexile AD 620L — Adult Directed — written for the adult voice in the room rather than for a child alone, with the mother carrying the explanations so the grown-up gets handed the script. You will know better than most how much that changes what has to happen on the page.
 Trade copies? I'll read yours properly and tell you the truth about it, which is the only thing worth trading.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -2050,8 +2050,8 @@
         <is>
           <t>Tom — you got more genuine engagement out of one post about kids and money than anyone else in this category has managed, which tells me you know exactly which part of this parents actually care about. I would like to check my premise against that.
 My premise: the whole field has the sequence backwards. Financial education starts children with saving. Saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it, standing in a store holding a birthday five, working out whether the thing is worth what it costs. We teach the second thing first and the first thing never.
-So I wrote and illustrated the spending book. Clarence Gets a Bargain follows one purchase the whole way , a boy wants a robot, earns it with chores and grades, reads the newspaper sale inserts at the kitchen table, compares two models on a shelf, takes the marked-down one on purpose, hands a coupon to the cashier, meets sales tax and objects to it, and then lives with what he chose. Idea to post-receipt; sixteen-plus concepts and nobody in the book says "budget." The reader works out he has been schooled only at the glossary , twenty-one terms in the back, page-referenced to the scene each came from. A jar is a storage container. It has never once talked a kid out of anything.
-The instruction underneath the whole book is four words long: stop bringing kids to the store as cargo, bring them as staff. Catalogued Lexile AD 620L , Adult Directed , so the parent gets handed the script rather than an assignment, which I suspect is why your posts land: parents want the conversation and do not feel qualified to start it.
+So I wrote and illustrated the spending book. Clarence Gets a Bargain follows one purchase the whole way — a boy wants a robot, earns it with chores and grades, reads the newspaper sale inserts at the kitchen table, compares two models on a shelf, takes the marked-down one on purpose, hands a coupon to the cashier, meets sales tax and objects to it, and then lives with what he chose. Idea to post-receipt; sixteen-plus concepts and nobody in the book says "budget." The reader works out he has been schooled only at the glossary — twenty-one terms in the back, page-referenced to the scene each came from. A jar is a storage container. It has never once talked a kid out of anything.
+The instruction underneath the whole book is four words long: stop bringing kids to the store as cargo, bring them as staff. Catalogued Lexile AD 620L — Adult Directed — so the parent gets handed the script rather than an assignment, which I suspect is why your posts land: parents want the conversation and do not feel qualified to start it.
 The thing I would actually value: you know what makes a parent stop scrolling on this subject and what makes them scroll past. If "spending before saving" is the wrong hook, I would rather hear it from you than keep testing it slowly.
 Would you look and tell me? https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -3079,8 +3079,8 @@
           <t>Stacy — you write about what happens to ordinary people inside financial systems. There is a version of that beat with no coverage at all, and it starts at about age six.
 A child becomes a consumer the first time they hand money to a cashier. Not at eighteen, not at a first paycheck — at six, with a birthday five. From that moment they are party to a transaction and they have rights nobody mentions: the receipt is proof, the price on the shelf has to match the price at the register, a broken thing can go back. Consumer education is the missing wing of children's financial literacy. We teach them to save and never tell them they are already the buyer.
 That is why I wrote the book. Clarence Gets a Bargain follows one purchase the entire way — a boy wants a robot, earns it, reads the sale inserts at the kitchen table, compares two on a shelf, takes the cheaper one on purpose, hands over a coupon, meets sales tax, and lives with what he chose. Idea to post-receipt; sixteen-plus concepts, none announced, and a twenty-one-term glossary in the back, each entry page-referenced to the scene it came from.
-The detail people ask me about: the mother photographs the receipt the second she sits down in the car. Every time. It takes four seconds and it is what makes a return, an exchange or a warranty claim winnable. Almost nobody teaches a child that, which is why the book is catalogued AD 620L , Adult Directed , and gets read with an adult rather than handed to a kid alone.
-I am an attorney, and on vacation that mostly means the souvenirs get cross-examined. The hermit crab: who feeds it over the holidays, and in two weeks when it dies , and buddy, it will , is it worth the tears? My kids find this insufferable. It is also the entire skill.
+The detail people ask me about: the mother photographs the receipt the second she sits down in the car. Every time. It takes four seconds and it is what makes a return, an exchange or a warranty claim winnable. Almost nobody teaches a child that, which is why the book is catalogued AD 620L — Adult Directed — and gets read with an adult rather than handed to a kid alone.
+I am an attorney, and on vacation that mostly means the souvenirs get cross-examined. The hermit crab: who feeds it over the holidays, and in two weeks when it dies — and buddy, it will — is it worth the tears? My kids find this insufferable. It is also the entire skill.
 The honest version of the beat problem: the full picture crosses agencies. Warranties and returns sit with the FTC, product safety with the CPSC. Nobody owns "children as consumers," which may be exactly why nobody covers it.
 Is there a story in that? clarencegetsabargain.com/press-kit.html
 Jonathan</t>
@@ -3633,8 +3633,8 @@
           <t>Prince — you took investing, which is the hardest concept in this category to make readable for children, and made it a series a kid comes back to. I went the opposite direction on the same shelf and I would like your read on it.
 Wesley learns to invest. Clarence learns to spend — and I mean the mechanics of it rather than the idea. Every other book in the category teaches saving, which is the second thing a child does with money. The first is spending, and a six-year-old has already done it, in a store, holding money, deciding whether the thing is worth what it costs. Nobody had written that one, so I did.
 Clarence Gets a Bargain follows a single purchase from beginning to end: a boy wants a robot, earns it with chores and grades, works the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one deliberately, hands a coupon to the cashier, meets sales tax, and then has to live with what he chose. Idea to post-receipt; sixteen-plus concepts, none of them announced. Nobody says the word "budget."
-The craft problem I would most like another author's view on: the reader is not supposed to know he has been taught anything until he reaches the glossary , twenty-one terms in the back, each page-referenced to the scene it came from. Getting that balance right, so it stays a story, was the whole job, and it is the thing most likely to be off by a hair. The rest of the shelf is piggy banks with plots. Good ones, some of them , but none of them has ever been to a register.
-I did the illustrations too, which means my opinion of them is worth nothing. It is written for the adult voice in the room , catalogued AD 620L, Adult Directed , with the mother carrying every explanation.
+The craft problem I would most like another author's view on: the reader is not supposed to know he has been taught anything until he reaches the glossary — twenty-one terms in the back, each page-referenced to the scene it came from. Getting that balance right, so it stays a story, was the whole job, and it is the thing most likely to be off by a hair. The rest of the shelf is piggy banks with plots. Good ones, some of them — but none of them has ever been to a register.
+I did the illustrations too, which means my opinion of them is worth nothing. It is written for the adult voice in the room — catalogued AD 620L, Adult Directed — with the mother carrying every explanation.
 Trade? Send me a Wesley and I will read it properly rather than politely.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -5776,9 +5776,9 @@
         <is>
           <t>Roda — you built a 30-Day Smart Spending Challenge. Not a saving challenge. Spending. As far as I can tell that makes two of us in this entire category who think the sequence is backwards.
 Here is my version of the argument, and I'd like to know whether it matches how you arrived at yours. Every children's money book teaches saving — I read all 25 on the ABA Foundation's list to be sure. But saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it, in a store, holding money, deciding whether the thing is worth what it costs. We teach the second thing first and the first thing never.
-Clarence Gets a Bargain is the picture-book version. It follows a single purchase the whole distance , a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he picked. Idea to post-receipt. Sixteen-plus concepts, none of them announced; nobody says "budget." Twenty-one terms in a glossary at the end, each page-referenced to where it happened , which is the only point at which a kid works out he's been schooled.
-One story takes a kid from "I want it" to "Is it worth it?" , which I suspect is the same door your Challenge walks them through, thirty days at a time. Yours is a habit; mine is one transaction read in twenty minutes. Those look complementary to me rather than competing , the book could be the on-ramp to a challenge, or the thing a parent reads on day one.
-One thing your Challenge and the book share: neither one works with a kid alone in a room. It is Lexile AD 620L , Adult Directed, the trade's code for read-with rather than read-alone , and the mother explains every concept on the page, so whoever is reading gets handed the script. Parent, teacher or grandparent, the reading stops every few pages because the kid asks something.
+Clarence Gets a Bargain is the picture-book version. It follows a single purchase the whole distance — a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he picked. Idea to post-receipt. Sixteen-plus concepts, none of them announced; nobody says "budget." Twenty-one terms in a glossary at the end, each page-referenced to where it happened — which is the only point at which a kid works out he's been schooled.
+One story takes a kid from "I want it" to "Is it worth it?" — which I suspect is the same door your Challenge walks them through, thirty days at a time. Yours is a habit; mine is one transaction read in twenty minutes. Those look complementary to me rather than competing — the book could be the on-ramp to a challenge, or the thing a parent reads on day one.
+One thing your Challenge and the book share: neither one works with a kid alone in a room. It is Lexile AD 620L — Adult Directed, the trade's code for read-with rather than read-alone — and the mother explains every concept on the page, so whoever is reading gets handed the script. Parent, teacher or grandparent, the reading stops every few pages because the kid asks something.
 Worth a conversation? I'd rather compare notes with the one other person who put spending first than pitch anybody.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -7108,8 +7108,8 @@
           <t>ML — you built a series a child comes back to, which is harder than writing one good book, and it's the reason I'm writing to a peer rather than a gatekeeper.
 Mine is a money book, which I appreciate is the least promising sentence in children's publishing. So here is the part that makes it not that.
 Every book in this category teaches saving. Saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it — in a store, holding money, deciding whether the thing is worth what it costs. So mine follows one purchase from the idea to after the receipt: a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he chose.
-The craft problem I'd most like another author's view on: I smuggled sixteen-plus concepts in without announcing any of them. Nobody says "budget." The glossary in the back , twenty-one terms, each page-referenced to the scene it came from , is the only place the book admits it was teaching. Getting that balance right, so it stays a story, was the whole job.
-The other half of the craft problem: it is written for an adult voice. Lexile AD 620L , Adult Directed , with the mother carrying every explanation, so whoever reads aloud gets handed the script. A series lives or dies on whether the grown-up still enjoys the fourth reading. You would know inside a page whether mine does.
+The craft problem I'd most like another author's view on: I smuggled sixteen-plus concepts in without announcing any of them. Nobody says "budget." The glossary in the back — twenty-one terms, each page-referenced to the scene it came from — is the only place the book admits it was teaching. Getting that balance right, so it stays a story, was the whole job.
+The other half of the craft problem: it is written for an adult voice. Lexile AD 620L — Adult Directed — with the mother carrying every explanation, so whoever reads aloud gets handed the script. A series lives or dies on whether the grown-up still enjoys the fourth reading. You would know inside a page whether mine does.
 Would you read it and tell me where it stops being a story? I'll trade — send me a Noah and I'll read it properly.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -17433,8 +17433,8 @@
           <t>Elizabeth — a scope question rather than a pitch.
 Federal attention to financial education, like every state mandate, concentrates on high school. Thirty states now require a course to graduate. The elementary standards that exist in most states sit underneath that with very little built against them, largely because nothing requires reporting at that band.
 The assumption underneath is that children begin with saving. Saving is the second thing a person does with money. The first is spending — a first grader has handled money at a register and made a decision there with no framework at all.
-I built a free, ungated K–5 resource for that: a 36-page picture book that follows one complete purchase from the idea through the receipt , sale ads, comparison shopping, a markdown, a coupon, sales tax , and a classroom set behind it. Four 45-minute lesson plans, a discussion guide, pre- and post-assessments with answer keys, printable classroom pieces, a browser-based pretend register, and a 23-row crosswalk to the 2021 National Standards for Personal Financial Education alongside Common Core Math and ELA, CEE and FDIC Money Smart, cited at the Grade 4 benchmark level rather than claimed generally. Sixteen-plus concepts appear in the story without being announced, and a twenty-one-term glossary in the back matter page-references each one to the scene where it occurs.
-No concept is announced in the text; the twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs. No account, no email capture, no purchase order. It prints from a browser. Catalogued Lexile AD 620L , Adult Directed , a one-period read-aloud requiring no instructor training.
+I built a free, ungated K–5 resource for that: a 36-page picture book that follows one complete purchase from the idea through the receipt — sale ads, comparison shopping, a markdown, a coupon, sales tax — and a classroom set behind it. Four 45-minute lesson plans, a discussion guide, pre- and post-assessments with answer keys, printable classroom pieces, a browser-based pretend register, and a 23-row crosswalk to the 2021 National Standards for Personal Financial Education alongside Common Core Math and ELA, CEE and FDIC Money Smart, cited at the Grade 4 benchmark level rather than claimed generally. Sixteen-plus concepts appear in the story without being announced, and a twenty-one-term glossary in the back matter page-references each one to the scene where it occurs.
+No concept is announced in the text; the twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs. No account, no email capture, no purchase order. It prints from a browser. Catalogued Lexile AD 620L — Adult Directed — a one-period read-aloud requiring no instructor training.
 The question: does any Department program or clearinghouse take elementary financial-education material, or is the practical route through the states? A steer on who would know is as useful to me as an answer.
 clarencegetsabargain.com/educator-toolkit.html
 Jonathan Bach
@@ -22046,9 +22046,9 @@
       <c r="K523" s="5" t="inlineStr">
         <is>
           <t>Ed — a narrow question about evidence standards, asked before I go further with something.
-I have built a free K–5 financial-education resource , a 36-page picture book plus a complete classroom set , and crosswalked it to the 2021 National Standards for Personal Financial Education, Common Core Math and ELA, CEE and FDIC Money Smart, at the Grade 4 benchmark level. Everything is ungated: no account, no email capture, no purchase order, and it prints from a browser.
+I have built a free K–5 financial-education resource — a 36-page picture book plus a complete classroom set — and crosswalked it to the 2021 National Standards for Personal Financial Education, Common Core Math and ELA, CEE and FDIC Money Smart, at the Grade 4 benchmark level. Everything is ungated: no account, no email capture, no purchase order, and it prints from a browser.
 The content premise is that the field has the sequence backwards. Financial education starts children with saving; saving is the second thing a person does with money. The first is spending, and a first grader has already done it at a register. The book follows one complete purchase from the idea through the receipt — the sale ads, the comparison, the markdown, the coupon, the sales tax, and living with what was bought. No concept is announced in the text; a twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs.
-One structural detail relevant to evaluation: the book is catalogued Lexile AD 620L , Adult Directed , so it is delivered as a shared read between an adult and a child rather than independent reading. That makes it closer to a shared-reading intervention than a curriculum, which may change what kind of evidence would be appropriate.
+One structural detail relevant to evaluation: the book is catalogued Lexile AD 620L — Adult Directed — so it is delivered as a shared read between an adult and a child rather than independent reading. That makes it closer to a shared-reading intervention than a curriculum, which may change what kind of evidence would be appropriate.
 The question: what would a resource like this need in order to be taken seriously on evidence — a pre/post instrument administered at scale, a quasi-experimental design, something else? I would rather build the right study once than assemble the wrong one. And if the honest answer is that no federal pathway exists for elementary material of this kind, that is worth knowing too.
 clarencegetsabargain.com/educator-toolkit.html
 Jonathan Bach
@@ -28613,8 +28613,8 @@
 Clarence Gets a Bargain carries a reading level of Lexile AD 620L. The AD stands for "Adult Directed" — the book industry's own label for a title meant to be read WITH a child rather than handed to one. That code isn't an accident. I built the book for the couch, not the corner.
 Here's why. In the story, Clarence doesn't learn about money from a worksheet. He learns it from his mom — at the kitchen table with the sale ads, in the car, in the middle of the store. Read the book to your kid and you aren't describing that scene. You're in it.
 And the interruptions will come. "Do we have a 529?" "Why do you take pictures of receipts?" "Can I hand the cashier the coupon next time?" "Is the internet a need or a want?" A kid alone in the corner reads a robot story and moves on. A kid pressed against your shoulder reads the same story and starts an argument about whether Wi-Fi counts as shelter. You want that argument. The argument is the product; the robot is the delivery vehicle.
-Every other money book for kids teaches saving, which is the second thing a child does with money. Spending is the first, and this one follows a single purchase the whole way , the sale ads, the aisle, the markdown, the coupon, the sales tax, and living with what got bought. Sixteen or more money concepts are in there and not one of them is announced. Nobody says the word "budget." Your kid won't know she's been taught anything until she reaches the glossary at the back , which is the last page, on purpose.
-You don't need to know anything about finance to do this well. Mom explains everything to Clarence inside the story , sale ads, clearance, markdowns, sales tax , so your only job is to read her lines like you knew it all along. I wrote you the script. Take the credit.
+Every other money book for kids teaches saving, which is the second thing a child does with money. Spending is the first, and this one follows a single purchase the whole way — the sale ads, the aisle, the markdown, the coupon, the sales tax, and living with what got bought. Sixteen or more money concepts are in there and not one of them is announced. Nobody says the word "budget." Your kid won't know she's been taught anything until she reaches the glossary at the back — which is the last page, on purpose.
+You don't need to know anything about finance to do this well. Mom explains everything to Clarence inside the story — sale ads, clearance, markdowns, sales tax — so your only job is to read her lines like you knew it all along. I wrote you the script. Take the credit.
 Two parts of the book flat-out require company:
 The grocery game, page 27. Whoever spots the biggest savings wins; the loser carries the bags in from the car. A kid cannot play this alone. That's the point.
 "Guess the Price," page 28. After dinner, somebody shares a deal they got that day and everyone guesses what it cost. Clarence guesses last and lowest, every time — his logic being that if a price is low enough to brag about at dinner, it has to be really low. Three players minimum. Grandma counts.
@@ -29033,9 +29033,9 @@
           <t>Kim — you review children's books for a living, so you have read more well-meaning money picture books than anyone should have to, and you already know the problem with them.
 They all teach saving. A piggy bank, a lemonade stand, a lesson. Which is fine advice in the wrong order, because saving is the second thing a child does with money; the first is spending. A six-year-old has no savings rate and has absolutely stood in a store holding money and had to decide.
 Mine is the spending one, and it follows a single purchase the whole distance rather than gesturing at the idea: a boy wants a robot, earns it with chores and grades, works the sale ads at the kitchen table, compares two models in the aisle, takes the cheaper one on purpose, hands a coupon to the cashier, gets hit with sales tax, and then has to live with the thing. Idea to post-receipt. I read all 25 on the ABA Foundation's list to be sure nobody had done it. Nobody had.
-What I'd actually want your eye on is the smuggling. Sixteen-plus concepts and not one of them is announced , no character stops to explain a term, nobody says "budget." The reader does not know he's been schooled until he reaches the glossary , twenty-one terms, each page-referenced to the scene it came from, working as a decoder rather than a homework appendix. The reveal is deliberate and it is on the last page. That balance is the hardest thing in the book and the thing most likely to be off by a hair.
+What I'd actually want your eye on is the smuggling. Sixteen-plus concepts and not one of them is announced — no character stops to explain a term, nobody says "budget." The reader does not know he's been schooled until he reaches the glossary — twenty-one terms, each page-referenced to the scene it came from, working as a decoder rather than a homework appendix. The reveal is deliberate and it is on the last page. That balance is the hardest thing in the book and the thing most likely to be off by a hair.
 One thing I'd want you to test rather than take on faith: whether it clicks later. The book is built to fire back months on, in a real store — "is the newer one really better? Clarence checked." Recognition first, then the habit. If that isn't actually in the pages, I'd want to know.
-The other thing worth your reviewer's ear: it is built to be read aloud, and Lexile has it at AD 620L — Adult Directed, read-with rather than read-alone. The mother carries the exposition, which means the adult holding the book is handed the script. Whether that voice actually holds up out loud , across a classroom, a couch, and a grandparent's lap , is something you would hear in a page and I can only guess at.
+The other thing worth your reviewer's ear: it is built to be read aloud, and Lexile has it at AD 620L — Adult Directed, read-with rather than read-alone. The mother carries the exposition, which means the adult holding the book is handed the script. Whether that voice actually holds up out loud — across a classroom, a couch, and a grandparent's lap — is something you would hear in a page and I can only guess at.
 Would you read it as an editor rather than as a friend? I would rather hear where it sags than be told it's charming.
 clarencegetsabargain.com/press-kit.html · https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -29277,9 +29277,9 @@
         <is>
           <t>Cinders — Moneybunnies splits money into Earn, Save, Spend and Give, which makes you the one person in this category who already agreed with me before I showed up.
 I went deep on one of your four. Spending, and specifically the whole transaction rather than the idea of it. Clarence Gets a Bargain follows a single purchase from beginning to end: a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then has to live with what he picked. Idea to post-receipt.
-The reason I think it sits beside Moneybunnies rather than against it: you give a child the four categories, and mine walks them through the mechanics of one. Sixteen-plus concepts, none announced , nobody says "budget" , and twenty-one terms in a glossary in the back, each page-referenced to the scene where it happened.
+The reason I think it sits beside Moneybunnies rather than against it: you give a child the four categories, and mine walks them through the mechanics of one. Sixteen-plus concepts, none announced — nobody says "budget" — and twenty-one terms in a glossary in the back, each page-referenced to the scene where it happened.
 Author-illustrator to author-illustrator: I did the art as well, so I know exactly how much of the work nobody sees. I'd rather you saw this from me than off a shelf.
-The read-aloud is the other half of it. Lexile AD 620L , Adult Directed , written for the adult voice in the room rather than for a child alone, with the mother carrying the explanations so the grown-up gets handed the script. You will know better than most how much that changes what has to happen on the page.
+The read-aloud is the other half of it. Lexile AD 620L — Adult Directed — written for the adult voice in the room rather than for a child alone, with the mother carrying the explanations so the grown-up gets handed the script. You will know better than most how much that changes what has to happen on the page.
 Trade copies? I'll read yours properly and tell you the truth about it, which is the only thing worth trading.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -30089,8 +30089,8 @@
         <is>
           <t>Tom — you got more genuine engagement out of one post about kids and money than anyone else in this category has managed, which tells me you know exactly which part of this parents actually care about. I would like to check my premise against that.
 My premise: the whole field has the sequence backwards. Financial education starts children with saving. Saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it, standing in a store holding a birthday five, working out whether the thing is worth what it costs. We teach the second thing first and the first thing never.
-So I wrote and illustrated the spending book. Clarence Gets a Bargain follows one purchase the whole way , a boy wants a robot, earns it with chores and grades, reads the newspaper sale inserts at the kitchen table, compares two models on a shelf, takes the marked-down one on purpose, hands a coupon to the cashier, meets sales tax and objects to it, and then lives with what he chose. Idea to post-receipt; sixteen-plus concepts and nobody in the book says "budget." The reader works out he has been schooled only at the glossary , twenty-one terms in the back, page-referenced to the scene each came from. A jar is a storage container. It has never once talked a kid out of anything.
-The instruction underneath the whole book is four words long: stop bringing kids to the store as cargo, bring them as staff. Catalogued Lexile AD 620L , Adult Directed , so the parent gets handed the script rather than an assignment, which I suspect is why your posts land: parents want the conversation and do not feel qualified to start it.
+So I wrote and illustrated the spending book. Clarence Gets a Bargain follows one purchase the whole way — a boy wants a robot, earns it with chores and grades, reads the newspaper sale inserts at the kitchen table, compares two models on a shelf, takes the marked-down one on purpose, hands a coupon to the cashier, meets sales tax and objects to it, and then lives with what he chose. Idea to post-receipt; sixteen-plus concepts and nobody in the book says "budget." The reader works out he has been schooled only at the glossary — twenty-one terms in the back, page-referenced to the scene each came from. A jar is a storage container. It has never once talked a kid out of anything.
+The instruction underneath the whole book is four words long: stop bringing kids to the store as cargo, bring them as staff. Catalogued Lexile AD 620L — Adult Directed — so the parent gets handed the script rather than an assignment, which I suspect is why your posts land: parents want the conversation and do not feel qualified to start it.
 The thing I would actually value: you know what makes a parent stop scrolling on this subject and what makes them scroll past. If "spending before saving" is the wrong hook, I would rather hear it from you than keep testing it slowly.
 Would you look and tell me? https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -31118,8 +31118,8 @@
           <t>Stacy — you write about what happens to ordinary people inside financial systems. There is a version of that beat with no coverage at all, and it starts at about age six.
 A child becomes a consumer the first time they hand money to a cashier. Not at eighteen, not at a first paycheck — at six, with a birthday five. From that moment they are party to a transaction and they have rights nobody mentions: the receipt is proof, the price on the shelf has to match the price at the register, a broken thing can go back. Consumer education is the missing wing of children's financial literacy. We teach them to save and never tell them they are already the buyer.
 That is why I wrote the book. Clarence Gets a Bargain follows one purchase the entire way — a boy wants a robot, earns it, reads the sale inserts at the kitchen table, compares two on a shelf, takes the cheaper one on purpose, hands over a coupon, meets sales tax, and lives with what he chose. Idea to post-receipt; sixteen-plus concepts, none announced, and a twenty-one-term glossary in the back, each entry page-referenced to the scene it came from.
-The detail people ask me about: the mother photographs the receipt the second she sits down in the car. Every time. It takes four seconds and it is what makes a return, an exchange or a warranty claim winnable. Almost nobody teaches a child that, which is why the book is catalogued AD 620L , Adult Directed , and gets read with an adult rather than handed to a kid alone.
-I am an attorney, and on vacation that mostly means the souvenirs get cross-examined. The hermit crab: who feeds it over the holidays, and in two weeks when it dies , and buddy, it will , is it worth the tears? My kids find this insufferable. It is also the entire skill.
+The detail people ask me about: the mother photographs the receipt the second she sits down in the car. Every time. It takes four seconds and it is what makes a return, an exchange or a warranty claim winnable. Almost nobody teaches a child that, which is why the book is catalogued AD 620L — Adult Directed — and gets read with an adult rather than handed to a kid alone.
+I am an attorney, and on vacation that mostly means the souvenirs get cross-examined. The hermit crab: who feeds it over the holidays, and in two weeks when it dies — and buddy, it will — is it worth the tears? My kids find this insufferable. It is also the entire skill.
 The honest version of the beat problem: the full picture crosses agencies. Warranties and returns sit with the FTC, product safety with the CPSC. Nobody owns "children as consumers," which may be exactly why nobody covers it.
 Is there a story in that? clarencegetsabargain.com/press-kit.html
 Jonathan</t>
@@ -31672,8 +31672,8 @@
           <t>Prince — you took investing, which is the hardest concept in this category to make readable for children, and made it a series a kid comes back to. I went the opposite direction on the same shelf and I would like your read on it.
 Wesley learns to invest. Clarence learns to spend — and I mean the mechanics of it rather than the idea. Every other book in the category teaches saving, which is the second thing a child does with money. The first is spending, and a six-year-old has already done it, in a store, holding money, deciding whether the thing is worth what it costs. Nobody had written that one, so I did.
 Clarence Gets a Bargain follows a single purchase from beginning to end: a boy wants a robot, earns it with chores and grades, works the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one deliberately, hands a coupon to the cashier, meets sales tax, and then has to live with what he chose. Idea to post-receipt; sixteen-plus concepts, none of them announced. Nobody says the word "budget."
-The craft problem I would most like another author's view on: the reader is not supposed to know he has been taught anything until he reaches the glossary , twenty-one terms in the back, each page-referenced to the scene it came from. Getting that balance right, so it stays a story, was the whole job, and it is the thing most likely to be off by a hair. The rest of the shelf is piggy banks with plots. Good ones, some of them , but none of them has ever been to a register.
-I did the illustrations too, which means my opinion of them is worth nothing. It is written for the adult voice in the room , catalogued AD 620L, Adult Directed , with the mother carrying every explanation.
+The craft problem I would most like another author's view on: the reader is not supposed to know he has been taught anything until he reaches the glossary — twenty-one terms in the back, each page-referenced to the scene it came from. Getting that balance right, so it stays a story, was the whole job, and it is the thing most likely to be off by a hair. The rest of the shelf is piggy banks with plots. Good ones, some of them — but none of them has ever been to a register.
+I did the illustrations too, which means my opinion of them is worth nothing. It is written for the adult voice in the room — catalogued AD 620L, Adult Directed — with the mother carrying every explanation.
 Trade? Send me a Wesley and I will read it properly rather than politely.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -31789,9 +31789,9 @@
         <is>
           <t>Roda — you built a 30-Day Smart Spending Challenge. Not a saving challenge. Spending. As far as I can tell that makes two of us in this entire category who think the sequence is backwards.
 Here is my version of the argument, and I'd like to know whether it matches how you arrived at yours. Every children's money book teaches saving — I read all 25 on the ABA Foundation's list to be sure. But saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it, in a store, holding money, deciding whether the thing is worth what it costs. We teach the second thing first and the first thing never.
-Clarence Gets a Bargain is the picture-book version. It follows a single purchase the whole distance , a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he picked. Idea to post-receipt. Sixteen-plus concepts, none of them announced; nobody says "budget." Twenty-one terms in a glossary at the end, each page-referenced to where it happened , which is the only point at which a kid works out he's been schooled.
-One story takes a kid from "I want it" to "Is it worth it?" , which I suspect is the same door your Challenge walks them through, thirty days at a time. Yours is a habit; mine is one transaction read in twenty minutes. Those look complementary to me rather than competing , the book could be the on-ramp to a challenge, or the thing a parent reads on day one.
-One thing your Challenge and the book share: neither one works with a kid alone in a room. It is Lexile AD 620L , Adult Directed, the trade's code for read-with rather than read-alone , and the mother explains every concept on the page, so whoever is reading gets handed the script. Parent, teacher or grandparent, the reading stops every few pages because the kid asks something.
+Clarence Gets a Bargain is the picture-book version. It follows a single purchase the whole distance — a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he picked. Idea to post-receipt. Sixteen-plus concepts, none of them announced; nobody says "budget." Twenty-one terms in a glossary at the end, each page-referenced to where it happened — which is the only point at which a kid works out he's been schooled.
+One story takes a kid from "I want it" to "Is it worth it?" — which I suspect is the same door your Challenge walks them through, thirty days at a time. Yours is a habit; mine is one transaction read in twenty minutes. Those look complementary to me rather than competing — the book could be the on-ramp to a challenge, or the thing a parent reads on day one.
+One thing your Challenge and the book share: neither one works with a kid alone in a room. It is Lexile AD 620L — Adult Directed, the trade's code for read-with rather than read-alone — and the mother explains every concept on the page, so whoever is reading gets handed the script. Parent, teacher or grandparent, the reading stops every few pages because the kid asks something.
 Worth a conversation? I'd rather compare notes with the one other person who put spending first than pitch anybody.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -31905,8 +31905,8 @@
           <t>ML — you built a series a child comes back to, which is harder than writing one good book, and it's the reason I'm writing to a peer rather than a gatekeeper.
 Mine is a money book, which I appreciate is the least promising sentence in children's publishing. So here is the part that makes it not that.
 Every book in this category teaches saving. Saving is the second thing a child does with money. The first is spending, and a six-year-old has already done it — in a store, holding money, deciding whether the thing is worth what it costs. So mine follows one purchase from the idea to after the receipt: a boy wants a robot, earns it with chores and grades, reads the sale inserts at the kitchen table, compares two models on a shelf, takes the cheaper one on purpose, hands a coupon to the cashier, meets sales tax, and then lives with what he chose.
-The craft problem I'd most like another author's view on: I smuggled sixteen-plus concepts in without announcing any of them. Nobody says "budget." The glossary in the back , twenty-one terms, each page-referenced to the scene it came from , is the only place the book admits it was teaching. Getting that balance right, so it stays a story, was the whole job.
-The other half of the craft problem: it is written for an adult voice. Lexile AD 620L , Adult Directed , with the mother carrying every explanation, so whoever reads aloud gets handed the script. A series lives or dies on whether the grown-up still enjoys the fourth reading. You would know inside a page whether mine does.
+The craft problem I'd most like another author's view on: I smuggled sixteen-plus concepts in without announcing any of them. Nobody says "budget." The glossary in the back — twenty-one terms, each page-referenced to the scene it came from — is the only place the book admits it was teaching. Getting that balance right, so it stays a story, was the whole job.
+The other half of the craft problem: it is written for an adult voice. Lexile AD 620L — Adult Directed — with the mother carrying every explanation, so whoever reads aloud gets handed the script. A series lives or dies on whether the grown-up still enjoys the fourth reading. You would know inside a page whether mine does.
 Would you read it and tell me where it stops being a story? I'll trade — send me a Noah and I'll read it properly.
 https://heyzine.com/flip-book/eeb1ef6cff.html
 Jonathan</t>
@@ -32458,8 +32458,8 @@
           <t>Elizabeth — a scope question rather than a pitch.
 Federal attention to financial education, like every state mandate, concentrates on high school. Thirty states now require a course to graduate. The elementary standards that exist in most states sit underneath that with very little built against them, largely because nothing requires reporting at that band.
 The assumption underneath is that children begin with saving. Saving is the second thing a person does with money. The first is spending — a first grader has handled money at a register and made a decision there with no framework at all.
-I built a free, ungated K–5 resource for that: a 36-page picture book that follows one complete purchase from the idea through the receipt , sale ads, comparison shopping, a markdown, a coupon, sales tax , and a classroom set behind it. Four 45-minute lesson plans, a discussion guide, pre- and post-assessments with answer keys, printable classroom pieces, a browser-based pretend register, and a 23-row crosswalk to the 2021 National Standards for Personal Financial Education alongside Common Core Math and ELA, CEE and FDIC Money Smart, cited at the Grade 4 benchmark level rather than claimed generally. Sixteen-plus concepts appear in the story without being announced, and a twenty-one-term glossary in the back matter page-references each one to the scene where it occurs.
-No concept is announced in the text; the twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs. No account, no email capture, no purchase order. It prints from a browser. Catalogued Lexile AD 620L , Adult Directed , a one-period read-aloud requiring no instructor training.
+I built a free, ungated K–5 resource for that: a 36-page picture book that follows one complete purchase from the idea through the receipt — sale ads, comparison shopping, a markdown, a coupon, sales tax — and a classroom set behind it. Four 45-minute lesson plans, a discussion guide, pre- and post-assessments with answer keys, printable classroom pieces, a browser-based pretend register, and a 23-row crosswalk to the 2021 National Standards for Personal Financial Education alongside Common Core Math and ELA, CEE and FDIC Money Smart, cited at the Grade 4 benchmark level rather than claimed generally. Sixteen-plus concepts appear in the story without being announced, and a twenty-one-term glossary in the back matter page-references each one to the scene where it occurs.
+No concept is announced in the text; the twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs. No account, no email capture, no purchase order. It prints from a browser. Catalogued Lexile AD 620L — Adult Directed — a one-period read-aloud requiring no instructor training.
 The question: does any Department program or clearinghouse take elementary financial-education material, or is the practical route through the states? A steer on who would know is as useful to me as an answer.
 clarencegetsabargain.com/educator-toolkit.html
 Jonathan Bach
@@ -32701,9 +32701,9 @@
       <c r="K66" s="5" t="inlineStr">
         <is>
           <t>Ed — a narrow question about evidence standards, asked before I go further with something.
-I have built a free K–5 financial-education resource , a 36-page picture book plus a complete classroom set , and crosswalked it to the 2021 National Standards for Personal Financial Education, Common Core Math and ELA, CEE and FDIC Money Smart, at the Grade 4 benchmark level. Everything is ungated: no account, no email capture, no purchase order, and it prints from a browser.
+I have built a free K–5 financial-education resource — a 36-page picture book plus a complete classroom set — and crosswalked it to the 2021 National Standards for Personal Financial Education, Common Core Math and ELA, CEE and FDIC Money Smart, at the Grade 4 benchmark level. Everything is ungated: no account, no email capture, no purchase order, and it prints from a browser.
 The content premise is that the field has the sequence backwards. Financial education starts children with saving; saving is the second thing a person does with money. The first is spending, and a first grader has already done it at a register. The book follows one complete purchase from the idea through the receipt — the sale ads, the comparison, the markdown, the coupon, the sales tax, and living with what was bought. No concept is announced in the text; a twenty-one-term glossary in the back matter carries the definitions, each page-referenced to where the term occurs.
-One structural detail relevant to evaluation: the book is catalogued Lexile AD 620L , Adult Directed , so it is delivered as a shared read between an adult and a child rather than independent reading. That makes it closer to a shared-reading intervention than a curriculum, which may change what kind of evidence would be appropriate.
+One structural detail relevant to evaluation: the book is catalogued Lexile AD 620L — Adult Directed — so it is delivered as a shared read between an adult and a child rather than independent reading. That makes it closer to a shared-reading intervention than a curriculum, which may change what kind of evidence would be appropriate.
 The question: what would a resource like this need in order to be taken seriously on evidence — a pre/post instrument administered at scale, a quasi-experimental design, something else? I would rather build the right study once than assemble the wrong one. And if the honest answer is that no federal pathway exists for elementary material of this kind, that is worth knowing too.
 clarencegetsabargain.com/educator-toolkit.html
 Jonathan Bach

</xml_diff>

<commit_message>
Add the missing subject line to the More Than Grand letter
GRAND carried one and More Than Grand did not, and both go out as email. The
subject mirrors the letter's hook, which is her own origin story: she built the
grandparent resource she could not find, same as he did on a different shelf.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bCVQmU5dQHBfkG189ujSG
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -28411,7 +28411,11 @@
           <t>deedee@morethangrand.com</t>
         </is>
       </c>
-      <c r="H667" s="5" t="inlineStr"/>
+      <c r="H667" s="5" t="inlineStr">
+        <is>
+          <t>You built the resource you couldn't find. So did I.</t>
+        </is>
+      </c>
       <c r="I667" s="5" t="n">
         <v>3162</v>
       </c>

</xml_diff>

<commit_message>
De-jargon 'crosswalked' in the one letter going to a journalist
Crosswalk is native vocabulary for curriculum directors, state finance offices,
Jump, CEE, NEFE, FDIC and superintendents, which is where 76 of the 77
uses land. The exception was Ben Eisen at the Wall Street Journal, where it
reads as inside baseball and costs a beat. Replaced with plain English.

Left Jennifer Klein's alone. Development officers read grant language daily and
'a standards crosswalk across five frameworks' is exactly what a funder wants
to see.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011bCVQmU5dQHBfkG189ujSG
</commit_message>
<xml_diff>
--- a/CGB_MASTER_outreach.xlsx
+++ b/CGB_MASTER_outreach.xlsx
@@ -3044,7 +3044,7 @@
           <t>Ben — a story pitch about a gap in the coverage rather than a book pitch, though the book is how I found it.
 Thirty states now guarantee a personal finance course. Every one of those mandates lands in high school. Money habits are largely set by seven, so the policy arrives roughly ten years after the cement dries — a fifteen-year-old handed a course for a habit he formed at six, and everyone acting surprised, and the funding, the training and the reporting all follow the mandate rather than the evidence.
 Underneath that sits an assumption nobody argues with: that children should learn saving first. I think it is backwards. Saving is the second thing a person does with money; the first is spending, and a first grader has done that, at a register, with a parent standing behind her. The behaviors a high school course tries to correct were installed a decade earlier by an arcade, a toy aisle and a checkout lane, none of which waited for a curriculum.
-I wrote the elementary piece rather than an op-ed about it. A 36-page picture book following one purchase from the idea to after the receipt — sale ads, comparison, a markdown, a coupon, sales tax, and living with the choice. Sixteen-plus concepts, none announced. A twenty-one-term glossary page-referenced into the story. Free ungated classroom set behind it, crosswalked to five frameworks. Catalogued Lexile AD 620L — Adult Directed, so it is a read-with, and the caregiver conversation happens inside the reading.
+I wrote the elementary piece rather than an op-ed about it. A 36-page picture book following one purchase from the idea to after the receipt — sale ads, comparison, a markdown, a coupon, sales tax, and living with the choice. Sixteen-plus concepts, none announced. A twenty-one-term glossary page-referenced into the story. Free ungated classroom set behind it, mapped concept by concept against the five standards frameworks states actually use. Catalogued Lexile AD 620L — Adult Directed, so it is a read-with, and the caregiver conversation happens inside the reading.
 Meanwhile the arcade never waited for a standard: $25 into a glass box for a basketball Walmart sells for $9.99, and the kid has no price memory to argue with.
 The story I would pitch your desk: the whole country legislated financial literacy into ninth grade, and the elementary standards that already exist in most states sit there with nothing built against them, because nobody has to report on them.
 Does that belong to anyone on your team? clarencegetsabargain.com/book-facts.html
@@ -31221,7 +31221,7 @@
           <t>Ben — a story pitch about a gap in the coverage rather than a book pitch, though the book is how I found it.
 Thirty states now guarantee a personal finance course. Every one of those mandates lands in high school. Money habits are largely set by seven, so the policy arrives roughly ten years after the cement dries — a fifteen-year-old handed a course for a habit he formed at six, and everyone acting surprised, and the funding, the training and the reporting all follow the mandate rather than the evidence.
 Underneath that sits an assumption nobody argues with: that children should learn saving first. I think it is backwards. Saving is the second thing a person does with money; the first is spending, and a first grader has done that, at a register, with a parent standing behind her. The behaviors a high school course tries to correct were installed a decade earlier by an arcade, a toy aisle and a checkout lane, none of which waited for a curriculum.
-I wrote the elementary piece rather than an op-ed about it. A 36-page picture book following one purchase from the idea to after the receipt — sale ads, comparison, a markdown, a coupon, sales tax, and living with the choice. Sixteen-plus concepts, none announced. A twenty-one-term glossary page-referenced into the story. Free ungated classroom set behind it, crosswalked to five frameworks. Catalogued Lexile AD 620L — Adult Directed, so it is a read-with, and the caregiver conversation happens inside the reading.
+I wrote the elementary piece rather than an op-ed about it. A 36-page picture book following one purchase from the idea to after the receipt — sale ads, comparison, a markdown, a coupon, sales tax, and living with the choice. Sixteen-plus concepts, none announced. A twenty-one-term glossary page-referenced into the story. Free ungated classroom set behind it, mapped concept by concept against the five standards frameworks states actually use. Catalogued Lexile AD 620L — Adult Directed, so it is a read-with, and the caregiver conversation happens inside the reading.
 Meanwhile the arcade never waited for a standard: $25 into a glass box for a basketball Walmart sells for $9.99, and the kid has no price memory to argue with.
 The story I would pitch your desk: the whole country legislated financial literacy into ninth grade, and the elementary standards that already exist in most states sit there with nothing built against them, because nobody has to report on them.
 Does that belong to anyone on your team? clarencegetsabargain.com/book-facts.html

</xml_diff>